<commit_message>
Fix auto-increment Excel error and push premium dashboard
</commit_message>
<xml_diff>
--- a/Estado_de_Cuenta_Flota.xlsx
+++ b/Estado_de_Cuenta_Flota.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Dueños" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Vehículos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Movimientos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Conductores" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Movimientos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -510,16 +511,16 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Generico</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>March</t>
+          <t>Vehiculo</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2020</v>
+        <v>2025</v>
       </c>
     </row>
   </sheetData>
@@ -533,6 +534,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Placa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Conductor Generico</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>UUO-808</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -1635,7 +1674,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>UUO-809</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1668,7 +1707,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>UUO-810</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1701,7 +1740,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>UUO-811</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1734,7 +1773,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>UUO-812</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1767,7 +1806,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>UUO-813</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1800,7 +1839,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>UUO-814</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1833,7 +1872,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>UUO-815</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1866,7 +1905,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>UUO-816</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1899,7 +1938,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>UUO-817</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1932,7 +1971,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>UUO-818</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1965,7 +2004,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>UUO-819</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1998,7 +2037,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>UUO-820</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2031,7 +2070,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>UUO-821</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2064,7 +2103,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>UUO-822</t>
+          <t>UUO-808</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">

</xml_diff>